<commit_message>
chore: utilise la clé Jira KAN-yy comme unique identifiant des stories
Remplace les identifiants US-xxx par les clés Jira KAN-yy dans le code
(commentaires uniquement), les tests, le contrat OpenAPI, la documentation,
les commandes Claude et les modèles GitHub. Supprime jira-mapping.md devenu
inutile. Les migrations Flyway V1 à V3, immuables, ne sont pas modifiées.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/backlog/Kadoo_Backlog_MVP_v1.2.xlsx
+++ b/docs/backlog/Kadoo_Backlog_MVP_v1.2.xlsx
@@ -311,7 +311,7 @@
     <t xml:space="preserve">L'Admin crée le partenaire (DRAFT), invite au moins un gestionnaire, définit le taux de commission, puis active le partenaire.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-002, US-004, US-005</t>
+    <t xml:space="preserve">KAN-18, KAN-21, KAN-22</t>
   </si>
   <si>
     <t xml:space="preserve">2 · Configuration</t>
@@ -320,7 +320,7 @@
     <t xml:space="preserve">Le gestionnaire crée une offre (valeur, prix, validité, conditions), son design et ses traductions ; fr-MA obligatoire.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-007, US-008, US-041, US-059</t>
+    <t xml:space="preserve">KAN-24, KAN-25, KAN-68, KAN-29</t>
   </si>
   <si>
     <t xml:space="preserve">3 · Distribution</t>
@@ -329,7 +329,7 @@
     <t xml:space="preserve">L'offre publiée apparaît au catalogue et est partagée par lien direct (UTM) ou bouton sur le site du partenaire.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-009, US-011, US-012, US-013</t>
+    <t xml:space="preserve">KAN-26, KAN-30, KAN-31, KAN-32</t>
   </si>
   <si>
     <t xml:space="preserve">4 · Achat</t>
@@ -338,7 +338,7 @@
     <t xml:space="preserve">L'acheteur (sans compte) choisit l'offre, le bénéficiaire, le canal, la langue et le message, puis accepte les CGV. Prix et taux sont figés.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-014 à US-017</t>
+    <t xml:space="preserve">KAN-33, KAN-34, KAN-35, KAN-36</t>
   </si>
   <si>
     <t xml:space="preserve">5 · Paiement</t>
@@ -347,7 +347,7 @@
     <t xml:space="preserve">Le PSP confirme le paiement par notification serveur signée ; la commande passe PAID ; la commission et la transaction sont enregistrées.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018, US-019, US-020, US-049</t>
+    <t xml:space="preserve">KAN-38, KAN-39, KAN-40, KAN-42</t>
   </si>
   <si>
     <t xml:space="preserve">6 · Émission et livraison</t>
@@ -356,7 +356,7 @@
     <t xml:space="preserve">Une carte unique est émise, puis envoyée par email ou partagée par WhatsApp ; l'acheteur reçoit sa confirmation.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-022 à US-025, US-036</t>
+    <t xml:space="preserve">KAN-44, KAN-45, KAN-46, KAN-47, KAN-63</t>
   </si>
   <si>
     <t xml:space="preserve">7 · Utilisation</t>
@@ -365,7 +365,7 @@
     <t xml:space="preserve">Le gestionnaire scanne le QR ou saisit le code, vérifie la carte, puis valide une utilisation unique et atomique.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-026, US-027</t>
+    <t xml:space="preserve">KAN-49, KAN-50</t>
   </si>
   <si>
     <t xml:space="preserve">8 · Pilotage</t>
@@ -374,7 +374,7 @@
     <t xml:space="preserve">Kadoo et le partenaire suivent ventes, utilisations, commissions et reversements.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-021, US-030, US-031, US-034</t>
+    <t xml:space="preserve">KAN-41, KAN-55, KAN-56, KAN-60</t>
   </si>
   <si>
     <t xml:space="preserve">RÈGLES TRANSVERSES</t>
@@ -569,7 +569,7 @@
     <t xml:space="preserve">Authentification et accès</t>
   </si>
   <si>
-    <t xml:space="preserve">US-001</t>
+    <t xml:space="preserve">KAN-17</t>
   </si>
   <si>
     <t xml:space="preserve">Connexion sécurisée</t>
@@ -605,13 +605,13 @@
     <t xml:space="preserve">À faire</t>
   </si>
   <si>
-    <t xml:space="preserve">US-038, US-039</t>
+    <t xml:space="preserve">KAN-65, KAN-66</t>
   </si>
   <si>
     <t xml:space="preserve">Réécrit</t>
   </si>
   <si>
-    <t xml:space="preserve">US-002</t>
+    <t xml:space="preserve">KAN-18</t>
   </si>
   <si>
     <t xml:space="preserve">Gérer les gestionnaires partenaires</t>
@@ -639,11 +639,11 @@
 AC4. Étant donné la liste des comptes, quand l'Admin filtre par partenaire et statut, alors seuls les comptes correspondants s'affichent.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-001, US-004, US-044
+    <t xml:space="preserve">KAN-17, KAN-21, KAN-71
 Persona corrigé (v1.0 : Admin / Partenaire).</t>
   </si>
   <si>
-    <t xml:space="preserve">US-003</t>
+    <t xml:space="preserve">KAN-19</t>
   </si>
   <si>
     <t xml:space="preserve">Réinitialiser son mot de passe</t>
@@ -668,10 +668,10 @@
 AC4. Étant donné un lien de plus de 30 min, alors il est refusé avec invitation à refaire une demande.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-001, US-044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-047</t>
+    <t xml:space="preserve">KAN-17, KAN-71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-20</t>
   </si>
   <si>
     <t xml:space="preserve">Double authentification Admin</t>
@@ -689,7 +689,7 @@
   </si>
   <si>
     <t xml:space="preserve">AC1. Étant donné un Admin sans MFA, quand il se connecte, alors il doit l'enrôler avant d'accéder au back-office.
-AC2. Étant donné un code TOTP invalide, alors l'accès est refusé et la tentative compte dans le verrouillage US-001.
+AC2. Étant donné un code TOTP invalide, alors l'accès est refusé et la tentative compte dans le verrouillage KAN-17.
 AC3. Étant donné un code de secours déjà utilisé, alors il est refusé.</t>
   </si>
   <si>
@@ -705,7 +705,7 @@
     <t xml:space="preserve">Gestion des partenaires</t>
   </si>
   <si>
-    <t xml:space="preserve">US-004</t>
+    <t xml:space="preserve">KAN-21</t>
   </si>
   <si>
     <t xml:space="preserve">Créer et activer un partenaire</t>
@@ -720,7 +720,7 @@
     <t xml:space="preserve">RG1. legalName, ICE, contactName et contactEmail obligatoires.
 RG2. ICE unique, 15 chiffres.
 RG3. RIB (24 chiffres) obligatoire à l'activation si Kadoo reverse les fonds (D-01).
-RG4. Activation possible seulement si : ≥ 1 gestionnaire invité, taux de commission actif (US-005), profil public fr-MA renseigné (US-006).
+RG4. Activation possible seulement si : ≥ 1 gestionnaire invité, taux de commission actif (KAN-22), profil public fr-MA renseigné (KAN-23).
 RG5. Seul un partenaire ACTIVE peut avoir des offres achetables.
 RG6. Toute modification est journalisée (valeur avant / après, hors RIB en clair).</t>
   </si>
@@ -731,14 +731,14 @@
 AC4. Étant donné tous les prérequis, quand l'Admin active, alors le statut passe ACTIVE et activatedAt est renseigné.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-002, US-005, US-006
+    <t xml:space="preserve">KAN-18, KAN-22, KAN-23
 Persona corrigé (v1.0 : Admin / Partenaire).</t>
   </si>
   <si>
     <t xml:space="preserve">D-01</t>
   </si>
   <si>
-    <t xml:space="preserve">US-005</t>
+    <t xml:space="preserve">KAN-22</t>
   </si>
   <si>
     <t xml:space="preserve">Configurer le taux de commission</t>
@@ -753,7 +753,7 @@
     <t xml:space="preserve">RG1. Taux compris entre 3,00 % et 10,00 %.
 RG2. Une seule période active à une date donnée (pas de chevauchement).
 RG3. effectiveFrom ≥ date du jour : aucune modification rétroactive.
-RG4. Le taux appliqué est celui actif à la création de la commande ; il est figé dans le snapshot de la commande puis repris dans la transaction (US-014, US-020).
+RG4. Le taux appliqué est celui actif à la création de la commande ; il est figé dans le snapshot de la commande puis repris dans la transaction (KAN-33, KAN-40).
 RG5. Historique conservé, non supprimable.</t>
   </si>
   <si>
@@ -763,14 +763,14 @@
 AC4. Étant donné une modification, alors l'historique affiche ancien taux, nouveau taux, auteur et date.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-004
+    <t xml:space="preserve">KAN-21
 Persona corrigé ; moment du figement précisé.</t>
   </si>
   <si>
     <t xml:space="preserve">D-02</t>
   </si>
   <si>
-    <t xml:space="preserve">US-006</t>
+    <t xml:space="preserve">KAN-23</t>
   </si>
   <si>
     <t xml:space="preserve">Personnaliser le profil public</t>
@@ -782,10 +782,10 @@
     <t xml:space="preserve">En tant que gestionnaire partenaire, je veux personnaliser le profil public de mon enseigne afin que les acheteurs la reconnaissent et lui fassent confiance.</t>
   </si>
   <si>
-    <t xml:space="preserve">PartnerProfile : partnerId, publicSlug, logoAssetId, bannerAssetId, websiteUrl, instagramUrl, city ; textes dans PartnerTranslation (US-042)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RG1. Images validées par US-059.
+    <t xml:space="preserve">PartnerProfile : partnerId, publicSlug, logoAssetId, bannerAssetId, websiteUrl, instagramUrl, city ; textes dans PartnerTranslation (KAN-69)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RG1. Images validées par KAN-29.
 RG2. URLs en https uniquement.
 RG3. Aucune donnée administrative exposée publiquement (ICE, RIB, contact interne, raison sociale si différente).
 RG4. publicSlug unique, généré à partir du nom commercial, modifiable par l'Admin uniquement.</t>
@@ -799,8 +799,8 @@
     <t xml:space="preserve">Lot 2</t>
   </si>
   <si>
-    <t xml:space="preserve">US-042, US-059
-Déplacé du Lot 1 au Lot 2 (dépend des médias US-059).</t>
+    <t xml:space="preserve">KAN-69, KAN-29
+Déplacé du Lot 1 au Lot 2 (dépend des médias KAN-29).</t>
   </si>
   <si>
     <t xml:space="preserve">EP03</t>
@@ -809,7 +809,7 @@
     <t xml:space="preserve">Offres et cartes</t>
   </si>
   <si>
-    <t xml:space="preserve">US-007</t>
+    <t xml:space="preserve">KAN-24</t>
   </si>
   <si>
     <t xml:space="preserve">Créer une offre en brouillon</t>
@@ -821,14 +821,14 @@
     <t xml:space="preserve">En tant que gestionnaire partenaire, je veux créer une offre de carte cadeau en brouillon afin de la préparer avant sa mise en vente.</t>
   </si>
   <si>
-    <t xml:space="preserve">Offer : id, partnerId, faceValue, salePrice, currency (MAD), validityDays, status, version, createdBy, updatedAt ; OfferTranslation (US-041)</t>
+    <t xml:space="preserve">Offer : id, partnerId, faceValue, salePrice, currency (MAD), validityDays, status, version, createdBy, updatedAt ; OfferTranslation (KAN-68)</t>
   </si>
   <si>
     <t xml:space="preserve">RG1. faceValue et salePrice &gt; 0, 2 décimales, entre 50 et 10 000 MAD (bornes D-12).
 RG2. salePrice ≤ faceValue ; hypothèse MVP : salePrice = faceValue (pas de remise).
 RG3. validityDays entre 30 et 730 jours, 365 par défaut.
 RG4. Devise MAD uniquement.
-RG5. Un brouillon peut être incomplet ; la publication exige la traduction fr-MA complète (titre, description, conditions, instructions) et un design (US-008).
+RG5. Un brouillon peut être incomplet ; la publication exige la traduction fr-MA complète (titre, description, conditions, instructions) et un design (KAN-25).
 RG6. L'offre n'est visible que par son partenaire et l'Admin.</t>
   </si>
   <si>
@@ -838,13 +838,13 @@
 AC4. Étant donné un gestionnaire d'un autre partenaire, alors l'offre lui est invisible.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-004, US-041</t>
+    <t xml:space="preserve">KAN-21, KAN-68</t>
   </si>
   <si>
     <t xml:space="preserve">D-12</t>
   </si>
   <si>
-    <t xml:space="preserve">US-008</t>
+    <t xml:space="preserve">KAN-25</t>
   </si>
   <si>
     <t xml:space="preserve">Personnaliser le design de la carte</t>
@@ -859,7 +859,7 @@
     <t xml:space="preserve">RG1. Couleurs au format HEX #RRGGBB.
 RG2. Contraste texte / fond ≥ 4,5:1 (WCAG AA) ; en dessous, avertissement bloquant à la publication.
 RG3. Aperçu mobile et desktop, en fr-MA et en ar-MA (RTL).
-RG4. Les cartes déjà émises gardent leur design (snapshot immuable, US-022).</t>
+RG4. Les cartes déjà émises gardent leur design (snapshot immuable, KAN-44).</t>
   </si>
   <si>
     <t xml:space="preserve">AC1. Étant donné un design enregistré, quand j'ouvre l'aperçu, alors je vois la carte en mobile et desktop, en français et en arabe.
@@ -867,10 +867,10 @@
 AC3. Étant donné une carte déjà émise, quand je modifie le design, alors la page cadeau de cette carte ne change pas.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-007, US-046, US-059</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-009</t>
+    <t xml:space="preserve">KAN-24, KAN-73, KAN-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-26</t>
   </si>
   <si>
     <t xml:space="preserve">Publier et dépublier une offre</t>
@@ -883,11 +883,11 @@
   </si>
   <si>
     <t xml:space="preserve">RG1. Transitions : DRAFT → PUBLISHED → UNPUBLISHED → PUBLISHED ; ARCHIVED est terminal (onglet 04).
-RG2. Publication possible si l'offre est complète (US-007) et le partenaire ACTIVE.
+RG2. Publication possible si l'offre est complète (KAN-24) et le partenaire ACTIVE.
 RG3. Une offre UNPUBLISHED n'accepte aucune nouvelle commande, y compris par lien direct.
 RG4. Une commande PENDING_PAYMENT créée avant la dépublication peut aboutir ; la carte est émise.
 RG5. Les cartes émises ne sont pas affectées.
-RG6. Si l'approbation Admin est retenue (D-04), la publication passe par US-055.</t>
+RG6. Si l'approbation Admin est retenue (D-04), la publication passe par KAN-28.</t>
   </si>
   <si>
     <t xml:space="preserve">AC1. Étant donné une offre incomplète, quand je publie, alors la publication est refusée avec la liste des éléments manquants.
@@ -896,13 +896,13 @@
 AC4. Étant donné une commande en attente de paiement au moment de la dépublication, quand le paiement est confirmé, alors la carte est émise normalement.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-007, US-008, US-041</t>
+    <t xml:space="preserve">KAN-24, KAN-25, KAN-68</t>
   </si>
   <si>
     <t xml:space="preserve">D-04</t>
   </si>
   <si>
-    <t xml:space="preserve">US-010</t>
+    <t xml:space="preserve">KAN-27</t>
   </si>
   <si>
     <t xml:space="preserve">Consulter et modifier ses offres</t>
@@ -925,7 +925,7 @@
 AC3. Étant donné une offre, quand je la duplique, alors une copie DRAFT est créée avec ses traductions et son design.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-055</t>
+    <t xml:space="preserve">KAN-28</t>
   </si>
   <si>
     <t xml:space="preserve">Approuver la publication d'une offre</t>
@@ -949,11 +949,11 @@
     <t xml:space="preserve">Lot 6</t>
   </si>
   <si>
-    <t xml:space="preserve">US-009, US-058
+    <t xml:space="preserve">KAN-26, KAN-62
 Conditionnelle : à supprimer si D-04 = publication autonome.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-059</t>
+    <t xml:space="preserve">KAN-29</t>
   </si>
   <si>
     <t xml:space="preserve">Téléverser et contrôler les médias</t>
@@ -979,7 +979,7 @@
 AC3. Étant donné une image valide, alors elle est disponible immédiatement pour le profil et le design.</t>
   </si>
   <si>
-    <t xml:space="preserve">Besoin implicite de US-006 et US-008 en v1.0.</t>
+    <t xml:space="preserve">Besoin implicite de KAN-23 et KAN-25 en v1.0.</t>
   </si>
   <si>
     <t xml:space="preserve">EP04</t>
@@ -988,7 +988,7 @@
     <t xml:space="preserve">Vitrine et distribution</t>
   </si>
   <si>
-    <t xml:space="preserve">US-011</t>
+    <t xml:space="preserve">KAN-30</t>
   </si>
   <si>
     <t xml:space="preserve">Consulter le catalogue</t>
@@ -1004,7 +1004,7 @@
   </si>
   <si>
     <t xml:space="preserve">RG1. Seules les offres PUBLISHED de partenaires ACTIVE sont visibles.
-RG2. Contenu affiché dans la langue courante avec fallback (US-045).
+RG2. Contenu affiché dans la langue courante avec fallback (KAN-72).
 RG3. Filtres MVP : ville et partenaire ; tri par prix et nouveauté.
 RG4. Montants formatés selon la locale (ex. 1 250,00 MAD).
 RG5. Aucun compte requis.</t>
@@ -1016,10 +1016,10 @@
 AC4. Étant donné une offre sans traduction en anglais, quand je navigue en anglais, alors le contenu fr-MA s'affiche.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-009, US-045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-012</t>
+    <t xml:space="preserve">KAN-26, KAN-72</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-31</t>
   </si>
   <si>
     <t xml:space="preserve">Partager le lien d'une offre</t>
@@ -1035,7 +1035,7 @@
   </si>
   <si>
     <t xml:space="preserve">RG1. Slug unique et stable dans le temps.
-RG2. Les paramètres UTM sont conservés jusqu'à la commande et enregistrés sur Order (BI US-030 / US-031).
+RG2. Les paramètres UTM sont conservés jusqu'à la commande et enregistrés sur Order (BI KAN-55 / KAN-56).
 RG3. Le lien d'une offre indisponible affiche une page « indisponible » avec les autres offres du partenaire.
 RG4. Balises Open Graph localisées (titre, image) pour l'aperçu WhatsApp, Instagram et Facebook.</t>
   </si>
@@ -1045,7 +1045,7 @@
 AC3. Étant donné une offre dépubliée, quand le lien est ouvert, alors l'achat est impossible.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-013</t>
+    <t xml:space="preserve">KAN-32</t>
   </si>
   <si>
     <t xml:space="preserve">Intégrer un bouton sur le site partenaire</t>
@@ -1065,8 +1065,8 @@
     <t xml:space="preserve">AC1. Étant donné le snippet collé sur une page, quand on clique, alors la bonne offre s'ouvre sur Kadoo avec utm_source=partner_site.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-012
-Repassée P1 : le lien partageable US-012 couvre le besoin du pilote.</t>
+    <t xml:space="preserve">KAN-31
+Repassée P1 : le lien partageable KAN-31 couvre le besoin du pilote.</t>
   </si>
   <si>
     <t xml:space="preserve">EP05</t>
@@ -1075,7 +1075,7 @@
     <t xml:space="preserve">Achat et personnalisation</t>
   </si>
   <si>
-    <t xml:space="preserve">US-014</t>
+    <t xml:space="preserve">KAN-33</t>
   </si>
   <si>
     <t xml:space="preserve">Initier une commande sans compte</t>
@@ -1092,7 +1092,7 @@
   <si>
     <t xml:space="preserve">RG1. L'offre doit être PUBLISHED et le partenaire ACTIVE au moment de la création.
 RG2. Prix, taux de commission, conditions et contenu de l'offre sont figés dans le snapshot.
-RG3. Statut initial PENDING_PAYMENT, expiration après 30 min (US-048).
+RG3. Statut initial PENDING_PAYMENT, expiration après 30 min (KAN-37).
 RG4. Référence unique non séquentielle (ex. KDO-2610-7Q4XK2).
 RG5. Email acheteur valide obligatoire ; une carte par commande.</t>
   </si>
@@ -1105,10 +1105,10 @@
     <t xml:space="preserve">Lot 3</t>
   </si>
   <si>
-    <t xml:space="preserve">US-009, US-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-015</t>
+    <t xml:space="preserve">KAN-26, KAN-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-34</t>
   </si>
   <si>
     <t xml:space="preserve">Renseigner le bénéficiaire</t>
@@ -1121,7 +1121,7 @@
   </si>
   <si>
     <t xml:space="preserve">RG1. Canal EMAIL : email bénéficiaire obligatoire et valide.
-RG2. Canal WHATSAPP : numéro facultatif ; le partage est fait par l'acheteur (US-025).
+RG2. Canal WHATSAPP : numéro facultatif ; le partage est fait par l'acheteur (KAN-47).
 RG3. Téléphone au format international, +212 proposé par défaut.
 RG4. Langue du bénéficiaire obligatoire, par défaut celle de l'acheteur.
 RG5. Seules les données nécessaires à la livraison sont collectées.</t>
@@ -1129,10 +1129,10 @@
   <si>
     <t xml:space="preserve">AC1. Étant donné le canal EMAIL sans email, alors le passage au paiement est bloqué avec un message sur le champ.
 AC2. Étant donné le numéro 0612345678, alors il est normalisé en +212612345678.
-AC3. Étant donné une langue bénéficiaire en arabe, alors la carte et l'email cadeau seront en arabe (US-043).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-016</t>
+AC3. Étant donné une langue bénéficiaire en arabe, alors la carte et l'email cadeau seront en arabe (KAN-70).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-35</t>
   </si>
   <si>
     <t xml:space="preserve">Ajouter un message personnel</t>
@@ -1155,7 +1155,7 @@
 AC3. Étant donné un message en arabe sur une carte en français, alors il s'affiche de droite à gauche dans son bloc.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-017</t>
+    <t xml:space="preserve">KAN-36</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmer le récapitulatif</t>
@@ -1168,7 +1168,7 @@
   </si>
   <si>
     <t xml:space="preserve">RG1. Le récapitulatif affiche : offre, partenaire, valeur, prix, date d'expiration prévisionnelle, conditions, bénéficiaire, canal, langue, message.
-RG2. Acceptation explicite des CGV (case non pré-cochée) ; la version acceptée est enregistrée (US-060).
+RG2. Acceptation explicite des CGV (case non pré-cochée) ; la version acceptée est enregistrée (KAN-76).
 RG3. Modification possible tant que le paiement n'est pas lancé.</t>
   </si>
   <si>
@@ -1177,10 +1177,10 @@
 AC3. Étant donné un retour en arrière, quand je corrige le bénéficiaire, alors le récapitulatif est mis à jour.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-015, US-016, US-060</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-048</t>
+    <t xml:space="preserve">KAN-34, KAN-35, KAN-76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-37</t>
   </si>
   <si>
     <t xml:space="preserve">Expirer les commandes non payées</t>
@@ -1195,9 +1195,9 @@
     <t xml:space="preserve">Order : status EXPIRED, expiresAt</t>
   </si>
   <si>
-    <t xml:space="preserve">RG1. Une commande PENDING_PAYMENT passe EXPIRED 30 min après sa création (paramètre US-058).
+    <t xml:space="preserve">RG1. Une commande PENDING_PAYMENT passe EXPIRED 30 min après sa création (paramètre KAN-62).
 RG2. Un paiement confirmé reçu après expiration est accepté : la commande passe PAID et la carte est émise (l'encaissement prime).
-RG3. Exception : si le partenaire est suspendu, la commande passe en remboursement (US-050).</t>
+RG3. Exception : si le partenaire est suspendu, la commande passe en remboursement (KAN-43).</t>
   </si>
   <si>
     <t xml:space="preserve">AC1. Étant donné une commande non payée depuis 31 min, alors elle est EXPIRED.
@@ -1205,7 +1205,7 @@
 AC3. Étant donné les KPI, alors les commandes EXPIRED ne comptent pas dans les ventes.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-014, US-018</t>
+    <t xml:space="preserve">KAN-33, KAN-38</t>
   </si>
   <si>
     <t xml:space="preserve">EP06</t>
@@ -1214,7 +1214,7 @@
     <t xml:space="preserve">Paiement et commissions</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018</t>
+    <t xml:space="preserve">KAN-38</t>
   </si>
   <si>
     <t xml:space="preserve">Payer en ligne via le PSP</t>
@@ -1246,7 +1246,7 @@
     <t xml:space="preserve">D-01, D-06</t>
   </si>
   <si>
-    <t xml:space="preserve">US-019</t>
+    <t xml:space="preserve">KAN-39</t>
   </si>
   <si>
     <t xml:space="preserve">Calculer la commission</t>
@@ -1270,10 +1270,10 @@
 AC3. Étant donné un changement de taux après la commande, alors le calcul utilise le taux figé.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-005, US-018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-020</t>
+    <t xml:space="preserve">KAN-22, KAN-38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-40</t>
   </si>
   <si>
     <t xml:space="preserve">Enregistrer la transaction financière</t>
@@ -1294,12 +1294,12 @@
 RG4. Remplace l'entité TransactionCommission de la v1.0 (fusion).</t>
   </si>
   <si>
-    <t xml:space="preserve">AC1. Étant donné un paiement confirmé, alors une transaction SALE RECORDED est créée avec les montants de US-019.
+    <t xml:space="preserve">AC1. Étant donné un paiement confirmé, alors une transaction SALE RECORDED est créée avec les montants de KAN-39.
 AC2. Étant donné une tentative de modification d'un montant, alors elle est refusée (y compris par l'Admin).
 AC3. Étant donné une recherche par providerTransactionId, alors la transaction et la commande associées s'affichent.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-021</t>
+    <t xml:space="preserve">KAN-41</t>
   </si>
   <si>
     <t xml:space="preserve">Suivre les reversements partenaires</t>
@@ -1325,14 +1325,14 @@
 AC4. Étant donné le dashboard partenaire, alors les montants dus et payés sont distincts.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-020
+    <t xml:space="preserve">KAN-40
 Repassée P1 / Lot 5 : premier reversement à la fin de la première période.</t>
   </si>
   <si>
     <t xml:space="preserve">D-01, D-02, D-11</t>
   </si>
   <si>
-    <t xml:space="preserve">US-049</t>
+    <t xml:space="preserve">KAN-42</t>
   </si>
   <si>
     <t xml:space="preserve">Rapprocher les paiements avec le PSP</t>
@@ -1345,7 +1345,7 @@
   </si>
   <si>
     <t xml:space="preserve">RG1. Toutes les 15 min : interrogation du PSP pour les paiements INITIATED de plus de 15 min.
-RG2. Un paiement confirmé chez le PSP mais pas chez Kadoo est traité comme une notification (même code idempotent que US-018).
+RG2. Un paiement confirmé chez le PSP mais pas chez Kadoo est traité comme une notification (même code idempotent que KAN-38).
 RG3. Rapport quotidien des anomalies : montant divergent, paiement inconnu, remboursement non tracé.
 RG4. Action Admin « resynchroniser » ; aucune saisie manuelle de statut de paiement.</t>
   </si>
@@ -1354,14 +1354,14 @@
 AC2. Étant donné un écart de montant, alors une anomalie est créée et visible par l'Admin.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018
+    <t xml:space="preserve">KAN-38
 Dépend de l'API de consultation du PSP choisi.</t>
   </si>
   <si>
     <t xml:space="preserve">D-06</t>
   </si>
   <si>
-    <t xml:space="preserve">US-050</t>
+    <t xml:space="preserve">KAN-43</t>
   </si>
   <si>
     <t xml:space="preserve">Rembourser une commande</t>
@@ -1376,7 +1376,7 @@
     <t xml:space="preserve">RG1. MVP : remboursement total exécuté dans le PSP (ou via son API), enregistré dans Kadoo avec motif.
 RG2. Impossible si la carte est REDEEMED.
 RG3. Effets : Order → REFUNDED, Payment → REFUNDED, carte → CANCELLED, écriture FinancialTransaction REFUND.
-RG4. Si la vente a déjà été reversée, le montant est déduit du reversement suivant (US-021).
+RG4. Si la vente a déjà été reversée, le montant est déduit du reversement suivant (KAN-41).
 RG5. Email de confirmation à l'acheteur.</t>
   </si>
   <si>
@@ -1385,7 +1385,7 @@
 AC3. Étant donné un remboursement, alors les KPI de ventes nettes diminuent du montant remboursé.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-020, US-051</t>
+    <t xml:space="preserve">KAN-40, KAN-53</t>
   </si>
   <si>
     <t xml:space="preserve">D-03</t>
@@ -1397,7 +1397,7 @@
     <t xml:space="preserve">Émission et livraison</t>
   </si>
   <si>
-    <t xml:space="preserve">US-022</t>
+    <t xml:space="preserve">KAN-44</t>
   </si>
   <si>
     <t xml:space="preserve">Émettre la carte cadeau</t>
@@ -1414,7 +1414,7 @@
 RG3. cardReference : identifiant public lisible (ex. KDO-7F3K-92QX), utilisé pour le support et l'historique.
 RG4. Code d'utilisation secret : 10 caractères sans ambiguïté (pas de 0/O, 1/I), généré par un générateur cryptographique, stocké uniquement sous forme de HMAC-SHA256 (recherche possible, jamais en clair).
 RG5. expiresAt = 23:59:59 heure du Maroc (Africa/Casablanca) du jour issuedAt + validityDays.
-RG6. Contenu figé dans la langue du bénéficiaire (US-043) et design figé (US-008).</t>
+RG6. Contenu figé dans la langue du bénéficiaire (KAN-70) et design figé (KAN-25).</t>
   </si>
   <si>
     <t xml:space="preserve">AC1. Étant donné un paiement confirmé, alors une carte ACTIVE est créée en moins de 10 s.
@@ -1426,10 +1426,10 @@
     <t xml:space="preserve">Lot 4</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018, US-043</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-023</t>
+    <t xml:space="preserve">KAN-38, KAN-70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-45</t>
   </si>
   <si>
     <t xml:space="preserve">Afficher la page cadeau</t>
@@ -1460,7 +1460,7 @@
     <t xml:space="preserve">D-05</t>
   </si>
   <si>
-    <t xml:space="preserve">US-024</t>
+    <t xml:space="preserve">KAN-46</t>
   </si>
   <si>
     <t xml:space="preserve">Envoyer la carte par email</t>
@@ -1472,7 +1472,7 @@
     <t xml:space="preserve">Delivery : giftCardId, channel, destination, locale, status (PENDING | SENT | FAILED | BOUNCED), attempts, providerMessageId, sentAt, lastError</t>
   </si>
   <si>
-    <t xml:space="preserve">RG1. Envoi asynchrone après émission, dans la langue du bénéficiaire (US-044).
+    <t xml:space="preserve">RG1. Envoi asynchrone après émission, dans la langue du bénéficiaire (KAN-71).
 RG2. 3 tentatives au maximum (après 1 min, 5 min, 30 min).
 RG3. Un échec d'envoi ne révoque jamais la carte ; l'Admin est alerté après le dernier échec.
 RG4. L'email contient le lien vers la page cadeau, pas le code en clair (D-15).
@@ -1484,13 +1484,13 @@
 AC3. Étant donné 3 échecs, alors Delivery = FAILED, la carte reste ACTIVE et l'Admin voit l'alerte.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-022, US-044</t>
+    <t xml:space="preserve">KAN-44, KAN-71</t>
   </si>
   <si>
     <t xml:space="preserve">D-15</t>
   </si>
   <si>
-    <t xml:space="preserve">US-025</t>
+    <t xml:space="preserve">KAN-47</t>
   </si>
   <si>
     <t xml:space="preserve">Partager la carte via WhatsApp</t>
@@ -1515,7 +1515,7 @@
     <t xml:space="preserve">D-07</t>
   </si>
   <si>
-    <t xml:space="preserve">US-053</t>
+    <t xml:space="preserve">KAN-48</t>
   </si>
   <si>
     <t xml:space="preserve">Renvoyer une carte ou corriger le destinataire</t>
@@ -1543,7 +1543,7 @@
     <t xml:space="preserve">Utilisation et contrôle</t>
   </si>
   <si>
-    <t xml:space="preserve">US-026</t>
+    <t xml:space="preserve">KAN-49</t>
   </si>
   <si>
     <t xml:space="preserve">Vérifier une carte en caisse</t>
@@ -1552,14 +1552,14 @@
     <t xml:space="preserve">En tant que gestionnaire partenaire, je veux scanner ou saisir le code d'une carte afin de savoir si elle est valable avant de fournir la prestation.</t>
   </si>
   <si>
-    <t xml:space="preserve">GiftCard : cardReference, partnerId, status, expiresAt, faceValue ; VerificationAttempt (US-052)</t>
+    <t xml:space="preserve">GiftCard : cardReference, partnerId, status, expiresAt, faceValue ; VerificationAttempt (KAN-54)</t>
   </si>
   <si>
     <t xml:space="preserve">RG1. Saisie manuelle du code ou scan du QR code depuis la caméra du téléphone (navigateur).
 RG2. La carte doit appartenir au partenaire du gestionnaire ; sinon, même message que pour un code inconnu (aucune fuite d'information).
 RG3. Affiche : statut, valeur, offre, date d'expiration, conditions, date d'utilisation si utilisée.
 RG4. La vérification ne consomme pas la carte ; elle est journalisée.
-RG5. L'expiration est contrôlée en temps réel (sans dépendre du traitement US-029).</t>
+RG5. L'expiration est contrôlée en temps réel (sans dépendre du traitement KAN-52).</t>
   </si>
   <si>
     <t xml:space="preserve">AC1. Étant donné une carte ACTIVE de mon partenaire, alors je vois sa valeur et le bouton « Valider l'utilisation ».
@@ -1568,10 +1568,10 @@
 AC4. Étant donné un QR code scanné, alors le résultat s'affiche en moins de 2 s.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-022, US-052</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-027</t>
+    <t xml:space="preserve">KAN-44, KAN-54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-50</t>
   </si>
   <si>
     <t xml:space="preserve">Valider l'utilisation d'une carte</t>
@@ -1587,7 +1587,7 @@
 RG2. Opération atomique : la carte passe REDEEMED seulement si elle est encore ACTIVE et non expirée ; contrainte unique sur giftCardId.
 RG3. Utilisation intégrale : pas de solde résiduel au MVP.
 RG4. Irréversible par le partenaire ; toute annulation passe par l'Admin.
-RG5. Déclenche la notification US-037.</t>
+RG5. Déclenche la notification KAN-64.</t>
   </si>
   <si>
     <t xml:space="preserve">AC1. Étant donné deux validations simultanées de la même carte, alors une seule réussit et l'autre affiche « déjà utilisée le … ».
@@ -1595,7 +1595,7 @@
 AC3. Étant donné une carte qui expire entre la vérification et la validation, alors la validation est refusée.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-028</t>
+    <t xml:space="preserve">KAN-51</t>
   </si>
   <si>
     <t xml:space="preserve">Consulter l'historique des utilisations</t>
@@ -1610,14 +1610,14 @@
     <t xml:space="preserve">RG1. Lecture limitée au partenaire connecté.
 RG2. Filtres : période, référence de carte, gestionnaire.
 RG3. Aucune suppression ni modification possible.
-RG4. Export via US-032.</t>
+RG4. Export via KAN-57.</t>
   </si>
   <si>
     <t xml:space="preserve">AC1. Étant donné une référence de carte, alors je retrouve son utilisation avec la date et le gestionnaire.
 AC2. Étant donné un filtre sur le mois en cours, alors seules les utilisations du mois s'affichent.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-029</t>
+    <t xml:space="preserve">KAN-52</t>
   </si>
   <si>
     <t xml:space="preserve">Expirer les cartes arrivées à échéance</t>
@@ -1630,7 +1630,7 @@
   </si>
   <si>
     <t xml:space="preserve">RG1. Traitement horaire : ACTIVE avec expiresAt dépassé → EXPIRED.
-RG2. Le refus d'utilisation après échéance est garanti par US-026 / US-027, même si le traitement n'est pas encore passé.
+RG2. Le refus d'utilisation après échéance est garanti par KAN-49 / KAN-50, même si le traitement n'est pas encore passé.
 RG3. Le sort des fonds des cartes expirées est défini par D-08.
 RG4. Option post-MVP : rappel au bénéficiaire 7 jours avant expiration.</t>
   </si>
@@ -1639,14 +1639,14 @@
 AC2. Étant donné une carte échue depuis 5 min, quand un gestionnaire la vérifie, alors elle est affichée comme expirée.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-022
+    <t xml:space="preserve">KAN-44
 Persona corrigé (v1.0 : Partenaire) : c'est un traitement système.</t>
   </si>
   <si>
     <t xml:space="preserve">D-08</t>
   </si>
   <si>
-    <t xml:space="preserve">US-051</t>
+    <t xml:space="preserve">KAN-53</t>
   </si>
   <si>
     <t xml:space="preserve">Bloquer ou annuler une carte</t>
@@ -1668,7 +1668,7 @@
 AC2. Étant donné une carte débloquée, alors elle redevient utilisable jusqu'à son expiration.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-052</t>
+    <t xml:space="preserve">KAN-54</t>
   </si>
   <si>
     <t xml:space="preserve">Protéger les codes contre la force brute</t>
@@ -1683,7 +1683,7 @@
     <t xml:space="preserve">RG1. 10 échecs en 15 min par gestionnaire, ou 30 par partenaire, bloquent la vérification 15 min.
 RG2. Alerte Admin en cas de blocage.
 RG3. Limitation équivalente sur l'accès aux pages cadeau (par IP).
-RG4. Code d'utilisation d'au moins 50 bits d'entropie (US-022).</t>
+RG4. Code d'utilisation d'au moins 50 bits d'entropie (KAN-44).</t>
   </si>
   <si>
     <t xml:space="preserve">AC1. Étant donné 10 codes invalides en 15 min, alors la 11e tentative est refusée pendant 15 min et l'Admin est alerté.
@@ -1696,7 +1696,7 @@
     <t xml:space="preserve">BI et reporting</t>
   </si>
   <si>
-    <t xml:space="preserve">US-030</t>
+    <t xml:space="preserve">KAN-55</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau de bord Admin</t>
@@ -1715,16 +1715,16 @@
 RG5. Chaque KPI a une définition affichée (info-bulle).</t>
   </si>
   <si>
-    <t xml:space="preserve">AC1. Étant donné une période, alors le total des ventes est égal à la somme des montants de l'export US-032 sur la même période.
+    <t xml:space="preserve">AC1. Étant donné une période, alors le total des ventes est égal à la somme des montants de l'export KAN-57 sur la même période.
 AC2. Étant donné un filtre partenaire, alors tous les KPI se limitent à ce partenaire.
 AC3. Étant donné une commande EXPIRED ou un paiement FAILED, alors ils ne comptent pas dans les ventes.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-020, US-027
-Repassée P1 : le suivi unitaire US-034 suffit au pilote ; à remonter en P0 si le pilote exige des KPI.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-031</t>
+    <t xml:space="preserve">KAN-40, KAN-50
+Repassée P1 : le suivi unitaire KAN-60 suffit au pilote ; à remonter en P0 si le pilote exige des KPI.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-56</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau de bord partenaire</t>
@@ -1738,18 +1738,18 @@
   <si>
     <t xml:space="preserve">RG1. Données limitées au partenaire connecté.
 RG2. Montants dus et montants reversés présentés séparément.
-RG3. Mêmes définitions que US-030.</t>
+RG3. Mêmes définitions que KAN-55.</t>
   </si>
   <si>
     <t xml:space="preserve">AC1. Étant donné un gestionnaire, alors aucun chiffre d'un autre partenaire n'est accessible, y compris via l'API.
 AC2. Étant donné une carte vendue puis utilisée, alors elle compte dans « émises » et « utilisées ».</t>
   </si>
   <si>
-    <t xml:space="preserve">US-030
+    <t xml:space="preserve">KAN-55
 Persona corrigé (v1.0 : Admin / Partenaire).</t>
   </si>
   <si>
-    <t xml:space="preserve">US-032</t>
+    <t xml:space="preserve">KAN-57</t>
   </si>
   <si>
     <t xml:space="preserve">Exporter les données en CSV</t>
@@ -1772,10 +1772,10 @@
 AC2. Étant donné un fichier ouvert dans Excel, alors les caractères arabes s'affichent correctement.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-030, US-031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-054</t>
+    <t xml:space="preserve">KAN-55, KAN-56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-58</t>
   </si>
   <si>
     <t xml:space="preserve">Consulter les ventes de mon partenaire</t>
@@ -1802,7 +1802,7 @@
     <t xml:space="preserve">Administration</t>
   </si>
   <si>
-    <t xml:space="preserve">US-033</t>
+    <t xml:space="preserve">KAN-59</t>
   </si>
   <si>
     <t xml:space="preserve">Superviser partenaires et offres</t>
@@ -1823,10 +1823,10 @@
 AC2. Étant donné une offre non conforme, quand l'Admin la dépublie avec un motif, alors elle n'est plus achetable et le partenaire voit le motif.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-004, US-009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-034</t>
+    <t xml:space="preserve">KAN-21, KAN-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-60</t>
   </si>
   <si>
     <t xml:space="preserve">Suivre commandes et paiements</t>
@@ -1847,10 +1847,10 @@
 AC2. Étant donné un paiement confirmé, alors aucun bouton ne permet d'en changer le statut ou le montant.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-038, US-022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-035</t>
+    <t xml:space="preserve">KAN-65, KAN-44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-61</t>
   </si>
   <si>
     <t xml:space="preserve">Suspendre un partenaire</t>
@@ -1864,7 +1864,7 @@
   <si>
     <t xml:space="preserve">RG1. Motif obligatoire ; action journalisée.
 RG2. Effet immédiat : aucune offre achetable, ni par le catalogue ni par lien direct.
-RG3. Une commande en attente payée après la suspension est remboursée (US-048, US-050).
+RG3. Une commande en attente payée après la suspension est remboursée (KAN-37, KAN-43).
 RG4. Hypothèse D-09 : les cartes ACTIVE restent utilisables ; le partenaire garde l'accès à la vérification et à la validation.
 RG5. Réactivation possible par l'Admin.</t>
   </si>
@@ -1876,7 +1876,7 @@
     <t xml:space="preserve">D-09</t>
   </si>
   <si>
-    <t xml:space="preserve">US-058</t>
+    <t xml:space="preserve">KAN-62</t>
   </si>
   <si>
     <t xml:space="preserve">Paramétrer les règles de la plateforme</t>
@@ -1901,7 +1901,7 @@
     <t xml:space="preserve">Notifications et audit</t>
   </si>
   <si>
-    <t xml:space="preserve">US-036</t>
+    <t xml:space="preserve">KAN-63</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmer l'achat à l'acheteur</t>
@@ -1923,11 +1923,11 @@
 AC2. Étant donné deux notifications PSP, alors un seul email est envoyé.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018, US-044
+    <t xml:space="preserve">KAN-38, KAN-71
 Déplacée du Lot 5 au Lot 4 : fait partie du parcours nominal.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-037</t>
+    <t xml:space="preserve">KAN-64</t>
   </si>
   <si>
     <t xml:space="preserve">Notifier l'utilisation</t>
@@ -1948,14 +1948,14 @@
 AC2. Étant donné une panne du service email, alors l'utilisation reste enregistrée.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-027, US-044
+    <t xml:space="preserve">KAN-50, KAN-71
 Destinataire de la notification précisé (absent en v1.0).</t>
   </si>
   <si>
     <t xml:space="preserve">D-13</t>
   </si>
   <si>
-    <t xml:space="preserve">US-038</t>
+    <t xml:space="preserve">KAN-65</t>
   </si>
   <si>
     <t xml:space="preserve">Journaliser les événements métier</t>
@@ -1983,7 +1983,7 @@
     <t xml:space="preserve">EP12</t>
   </si>
   <si>
-    <t xml:space="preserve">US-039</t>
+    <t xml:space="preserve">KAN-66</t>
   </si>
   <si>
     <t xml:space="preserve">Configurer les langues</t>
@@ -2007,7 +2007,7 @@
     <t xml:space="preserve">Persona corrigé (v1.0 : Tous / Partenaire / Système).</t>
   </si>
   <si>
-    <t xml:space="preserve">US-040</t>
+    <t xml:space="preserve">KAN-67</t>
   </si>
   <si>
     <t xml:space="preserve">Changer la langue de l'interface</t>
@@ -2056,7 +2056,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">US-041</t>
+    <t xml:space="preserve">KAN-68</t>
   </si>
   <si>
     <t xml:space="preserve">Traduire une offre</t>
@@ -2078,10 +2078,10 @@
 AC2. Étant donné une traduction ar-MA, alors le formulaire de saisie est en RTL.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-007, US-045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-042</t>
+    <t xml:space="preserve">KAN-24, KAN-72</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-69</t>
   </si>
   <si>
     <t xml:space="preserve">Traduire le profil partenaire</t>
@@ -2100,10 +2100,10 @@
     <t xml:space="preserve">AC1. Étant donné un profil traduit en arabe, alors un visiteur en arabe voit le nom et la description arabes.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-006, US-045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-043</t>
+    <t xml:space="preserve">KAN-23, KAN-72</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-70</t>
   </si>
   <si>
     <t xml:space="preserve">Carte dans la langue du bénéficiaire</t>
@@ -2116,7 +2116,7 @@
   </si>
   <si>
     <t xml:space="preserve">RG1. La langue de l'acheteur et celle du bénéficiaire sont indépendantes.
-RG2. Le contenu de l'offre est figé dans la langue du bénéficiaire à l'émission (avec fallback US-045).
+RG2. Le contenu de l'offre est figé dans la langue du bénéficiaire à l'émission (avec fallback KAN-72).
 RG3. Le message personnel n'est pas traduit.</t>
   </si>
   <si>
@@ -2124,10 +2124,10 @@
 AC2. Étant donné une traduction modifiée après émission, alors la carte émise ne change pas.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-022, US-041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-044</t>
+    <t xml:space="preserve">KAN-44, KAN-68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-71</t>
   </si>
   <si>
     <t xml:space="preserve">Modèles de notifications localisés</t>
@@ -2139,7 +2139,7 @@
     <t xml:space="preserve">NotificationTemplate : eventType, locale, subject, bodyHtml, bodyText, version</t>
   </si>
   <si>
-    <t xml:space="preserve">RG1. Un modèle par (eventType, locale) ; fr-MA obligatoire, fallback US-045.
+    <t xml:space="preserve">RG1. Un modèle par (eventType, locale) ; fr-MA obligatoire, fallback KAN-72.
 RG2. Achat → langue acheteur ; cadeau → langue bénéficiaire ; back-office → préférence utilisateur.
 RG3. Variables échappées ; emails arabes en RTL.
 RG4. Événements : invitation, réinitialisation, achat confirmé, carte cadeau, utilisation, remboursement.</t>
@@ -2149,11 +2149,11 @@
 AC2. Étant donné un nom d'acheteur contenant du HTML, alors il s'affiche comme du texte.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-039, US-045
-Déplacée du Lot 4 au Lot 1 : US-002 et US-003 envoient des emails dès le Lot 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-045</t>
+    <t xml:space="preserve">KAN-66, KAN-72
+Déplacée du Lot 4 au Lot 1 : KAN-18 et KAN-19 envoient des emails dès le Lot 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-72</t>
   </si>
   <si>
     <t xml:space="preserve">Repli sur une langue disponible</t>
@@ -2172,7 +2172,7 @@
     <t xml:space="preserve">AC1. Étant donné une offre sans traduction anglaise, quand un visiteur l'ouvre en anglais, alors le contenu fr-MA s'affiche et l'interface reste en anglais.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-046</t>
+    <t xml:space="preserve">KAN-73</t>
   </si>
   <si>
     <t xml:space="preserve">Affichage arabe de droite à gauche</t>
@@ -2193,7 +2193,7 @@
 AC2. Étant donné une référence KDO-7F3K-92QX dans une phrase arabe, alors elle s'affiche dans le bon ordre.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-039
+    <t xml:space="preserve">KAN-66
 Effort transverse : chaque US d'interface inclut sa recette RTL.</t>
   </si>
   <si>
@@ -2203,7 +2203,7 @@
     <t xml:space="preserve">Conformité et protection des données</t>
   </si>
   <si>
-    <t xml:space="preserve">US-056</t>
+    <t xml:space="preserve">KAN-74</t>
   </si>
   <si>
     <t xml:space="preserve">Informer et recueillir le consentement (loi 09-08)</t>
@@ -2229,13 +2229,13 @@
 AC2. Étant donné la page cadeau, alors une mention indique l'origine des données et le lien vers la politique.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-060</t>
+    <t xml:space="preserve">KAN-76</t>
   </si>
   <si>
     <t xml:space="preserve">D-10</t>
   </si>
   <si>
-    <t xml:space="preserve">US-057</t>
+    <t xml:space="preserve">KAN-75</t>
   </si>
   <si>
     <t xml:space="preserve">Conserver puis anonymiser les données</t>
@@ -2265,7 +2265,7 @@
   </si>
   <si>
     <t xml:space="preserve">RG1. Documents en 3 langues, versionnés ; une seule version en vigueur par type.
-RG2. La version des CGV acceptée est enregistrée sur chaque commande (US-017).
+RG2. La version des CGV acceptée est enregistrée sur chaque commande (KAN-36).
 RG3. Souvent exigé par le PSP pour l'activation du compte marchand.</t>
   </si>
   <si>
@@ -2326,7 +2326,7 @@
     <t xml:space="preserve">Suspension</t>
   </si>
   <si>
-    <t xml:space="preserve">Motif obligatoire ; offres non achetables ; cartes selon D-09 (US-035).</t>
+    <t xml:space="preserve">Motif obligatoire ; offres non achetables ; cartes selon D-09 (KAN-61).</t>
   </si>
   <si>
     <t xml:space="preserve">Réactivation</t>
@@ -2356,7 +2356,7 @@
     <t xml:space="preserve">Invitation</t>
   </si>
   <si>
-    <t xml:space="preserve">Jeton valable 72 h (US-002).</t>
+    <t xml:space="preserve">Jeton valable 72 h (KAN-18).</t>
   </si>
   <si>
     <t xml:space="preserve">Acceptation de l'invitation</t>
@@ -2401,7 +2401,7 @@
     <t xml:space="preserve">Soumission</t>
   </si>
   <si>
-    <t xml:space="preserve">Uniquement si approbation Admin (US-055).</t>
+    <t xml:space="preserve">Uniquement si approbation Admin (KAN-28).</t>
   </si>
   <si>
     <t xml:space="preserve">PUBLISHED / DRAFT</t>
@@ -2464,7 +2464,7 @@
     <t xml:space="preserve">TTL dépassé</t>
   </si>
   <si>
-    <t xml:space="preserve">US-048.</t>
+    <t xml:space="preserve">KAN-37.</t>
   </si>
   <si>
     <t xml:space="preserve">Paiement confirmé tardif</t>
@@ -2482,7 +2482,7 @@
     <t xml:space="preserve">Remboursement</t>
   </si>
   <si>
-    <t xml:space="preserve">Carte non utilisée ; carte → CANCELLED (US-050).</t>
+    <t xml:space="preserve">Carte non utilisée ; carte → CANCELLED (KAN-43).</t>
   </si>
   <si>
     <t xml:space="preserve">Payment</t>
@@ -2521,13 +2521,13 @@
     <t xml:space="preserve">Nouvelle tentative possible.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-050.</t>
+    <t xml:space="preserve">KAN-43.</t>
   </si>
   <si>
     <t xml:space="preserve">GiftCard</t>
   </si>
   <si>
-    <t xml:space="preserve">Une carte par commande (US-022).</t>
+    <t xml:space="preserve">Une carte par commande (KAN-44).</t>
   </si>
   <si>
     <t xml:space="preserve">REDEEMED</t>
@@ -2536,13 +2536,13 @@
     <t xml:space="preserve">Validation de l'utilisation</t>
   </si>
   <si>
-    <t xml:space="preserve">Atomique ; terminal (US-027).</t>
+    <t xml:space="preserve">Atomique ; terminal (KAN-50).</t>
   </si>
   <si>
     <t xml:space="preserve">Échéance dépassée</t>
   </si>
   <si>
-    <t xml:space="preserve">Terminal au MVP (US-029, D-08).</t>
+    <t xml:space="preserve">Terminal au MVP (KAN-52, D-08).</t>
   </si>
   <si>
     <t xml:space="preserve">BLOCKED</t>
@@ -2551,7 +2551,7 @@
     <t xml:space="preserve">Suspicion de fraude</t>
   </si>
   <si>
-    <t xml:space="preserve">Réversible (US-051).</t>
+    <t xml:space="preserve">Réversible (KAN-53).</t>
   </si>
   <si>
     <t xml:space="preserve">Déblocage</t>
@@ -2566,7 +2566,7 @@
     <t xml:space="preserve">CANCELLED</t>
   </si>
   <si>
-    <t xml:space="preserve">Terminal (US-050).</t>
+    <t xml:space="preserve">Terminal (KAN-43).</t>
   </si>
   <si>
     <t xml:space="preserve">Delivery (email)</t>
@@ -2578,7 +2578,7 @@
     <t xml:space="preserve">Émission de la carte</t>
   </si>
   <si>
-    <t xml:space="preserve">US-024.</t>
+    <t xml:space="preserve">KAN-46.</t>
   </si>
   <si>
     <t xml:space="preserve">SENT</t>
@@ -2605,7 +2605,7 @@
     <t xml:space="preserve">Service email</t>
   </si>
   <si>
-    <t xml:space="preserve">Alerte support (US-053).</t>
+    <t xml:space="preserve">Alerte support (KAN-48).</t>
   </si>
   <si>
     <t xml:space="preserve">Delivery (WhatsApp)</t>
@@ -2617,7 +2617,7 @@
     <t xml:space="preserve">Affichage du bouton</t>
   </si>
   <si>
-    <t xml:space="preserve">US-025.</t>
+    <t xml:space="preserve">KAN-47.</t>
   </si>
   <si>
     <t xml:space="preserve">LINK_OPENED</t>
@@ -2638,7 +2638,7 @@
     <t xml:space="preserve">Paiement confirmé</t>
   </si>
   <si>
-    <t xml:space="preserve">Type SALE (US-020).</t>
+    <t xml:space="preserve">Type SALE (KAN-40).</t>
   </si>
   <si>
     <t xml:space="preserve">SETTLED</t>
@@ -2647,7 +2647,7 @@
     <t xml:space="preserve">Reversement PAID</t>
   </si>
   <si>
-    <t xml:space="preserve">US-021.</t>
+    <t xml:space="preserve">KAN-41.</t>
   </si>
   <si>
     <t xml:space="preserve">REVERSED</t>
@@ -2752,7 +2752,7 @@
     <t xml:space="preserve">tokenHash unique</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouveau (US-002)</t>
+    <t xml:space="preserve">Nouveau (KAN-18)</t>
   </si>
   <si>
     <t xml:space="preserve">PasswordResetToken</t>
@@ -2761,7 +2761,7 @@
     <t xml:space="preserve">id, userId, tokenHash, expiresAt, usedAt</t>
   </si>
   <si>
-    <t xml:space="preserve">Ajouté au modèle (cité en US-003)</t>
+    <t xml:space="preserve">Ajouté au modèle (cité en KAN-19)</t>
   </si>
   <si>
     <t xml:space="preserve">id, legalName, tradeName, ICE, contactName, contactEmail, phone, city, address, bankRib (chiffré), status, activatedAt, suspensionReason, suspendedAt</t>
@@ -2788,7 +2788,7 @@
     <t xml:space="preserve">publicSlug unique</t>
   </si>
   <si>
-    <t xml:space="preserve">Ajouté au modèle (cité en US-006)</t>
+    <t xml:space="preserve">Ajouté au modèle (cité en KAN-23)</t>
   </si>
   <si>
     <t xml:space="preserve">PartnerTranslation</t>
@@ -2812,7 +2812,7 @@
     <t xml:space="preserve">pas de chevauchement de périodes ; 3 ≤ rate ≤ 10</t>
   </si>
   <si>
-    <t xml:space="preserve">Ajouté au modèle (cité en US-005)</t>
+    <t xml:space="preserve">Ajouté au modèle (cité en KAN-22)</t>
   </si>
   <si>
     <t xml:space="preserve">MediaAsset</t>
@@ -2821,7 +2821,7 @@
     <t xml:space="preserve">id, partnerId, type, mimeType, sizeBytes, width, height, storageKey</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouveau (US-059)</t>
+    <t xml:space="preserve">Nouveau (KAN-29)</t>
   </si>
   <si>
     <t xml:space="preserve">id, partnerId, faceValue, salePrice, currency, validityDays, status, version, publishedAt, unpublishedAt</t>
@@ -2944,7 +2944,7 @@
     <t xml:space="preserve">≤ 1 par Order au MVP (remboursement total)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouveau (US-050)</t>
+    <t xml:space="preserve">Nouveau (KAN-43)</t>
   </si>
   <si>
     <t xml:space="preserve">id, orderId, paymentId, partnerId, type, grossAmount, commissionRate, commissionAmount, partnerAmount, currency, status, settlementId</t>
@@ -2992,7 +2992,7 @@
     <t xml:space="preserve">publicTokenHash unique</t>
   </si>
   <si>
-    <t xml:space="preserve">Ajouté au modèle (cité en US-023)</t>
+    <t xml:space="preserve">Ajouté au modèle (cité en KAN-45)</t>
   </si>
   <si>
     <t xml:space="preserve">Redemption</t>
@@ -3013,7 +3013,7 @@
     <t xml:space="preserve">index (userId, occurredAt)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouveau (US-052)</t>
+    <t xml:space="preserve">Nouveau (KAN-54)</t>
   </si>
   <si>
     <t xml:space="preserve">Delivery</t>
@@ -3037,7 +3037,7 @@
     <t xml:space="preserve">unique (eventType, eventId) : idempotence</t>
   </si>
   <si>
-    <t xml:space="preserve">Ajouté au modèle (cité en US-036/037)</t>
+    <t xml:space="preserve">Ajouté au modèle (cité en KAN-63/037)</t>
   </si>
   <si>
     <t xml:space="preserve">NotificationTemplate</t>
@@ -3058,7 +3058,7 @@
     <t xml:space="preserve">N:1 Payment</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouveau (US-049)</t>
+    <t xml:space="preserve">Nouveau (KAN-42)</t>
   </si>
   <si>
     <t xml:space="preserve">LegalDocument</t>
@@ -3070,7 +3070,7 @@
     <t xml:space="preserve">une version en vigueur par (type, locale)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouveau (US-060)</t>
+    <t xml:space="preserve">Nouveau (KAN-76)</t>
   </si>
   <si>
     <t xml:space="preserve">PlatformSetting</t>
@@ -3082,7 +3082,7 @@
     <t xml:space="preserve">PK key</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouveau (US-058)</t>
+    <t xml:space="preserve">Nouveau (KAN-62)</t>
   </si>
   <si>
     <t xml:space="preserve">AuditEvent</t>
@@ -3142,10 +3142,10 @@
     <t xml:space="preserve">A. Kadoo encaisse puis reverse • B. Le partenaire encaisse et paie la commission • C. Paiement fractionné par le PSP</t>
   </si>
   <si>
-    <t xml:space="preserve">A pour le MVP (cohérent avec US-021 et le reversement manuel), sous réserve de validation juridique : encaisser pour compte de tiers peut relever d'un statut réglementé (Bank Al-Maghrib). À défaut, C si le PSP le permet.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-004, US-018, US-019, US-020, US-021</t>
+    <t xml:space="preserve">A pour le MVP (cohérent avec KAN-41 et le reversement manuel), sous réserve de validation juridique : encaisser pour compte de tiers peut relever d'un statut réglementé (Bank Al-Maghrib). À défaut, C si le PSP le permet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-21, KAN-38, KAN-39, KAN-40, KAN-41</t>
   </si>
   <si>
     <t xml:space="preserve">Direction / Juridique / Finance</t>
@@ -3166,7 +3166,7 @@
     <t xml:space="preserve">Base = montant payé TTC ; commission facturée au partenaire (HT + TVA) mensuellement ; frais PSP supportés par Kadoo (inclus dans le taux). Périodicité de reversement : mensuelle.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-005, US-019, US-021, US-030, US-031, US-036</t>
+    <t xml:space="preserve">KAN-22, KAN-39, KAN-41, KAN-55, KAN-56, KAN-63</t>
   </si>
   <si>
     <t xml:space="preserve">Finance / Expert-comptable</t>
@@ -3181,10 +3181,10 @@
     <t xml:space="preserve">Manuel encadré par l'Admin • workflow intégré • aucun remboursement</t>
   </si>
   <si>
-    <t xml:space="preserve">Manuel encadré au MVP : total uniquement, carte non utilisée, motif obligatoire (US-050). Vérifier l'application du droit de rétractation de la loi 31-08 aux cartes cadeaux.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-050, US-051, US-060</t>
+    <t xml:space="preserve">Manuel encadré au MVP : total uniquement, carte non utilisée, motif obligatoire (KAN-43). Vérifier l'application du droit de rétractation de la loi 31-08 aux cartes cadeaux.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-43, KAN-53, KAN-76</t>
   </si>
   <si>
     <t xml:space="preserve">Juridique / Produit</t>
@@ -3199,10 +3199,10 @@
     <t xml:space="preserve">Autonome • approbation Admin</t>
   </si>
   <si>
-    <t xml:space="preserve">Autonome au MVP : les partenaires sont onboardés à la main (contrôle à l'entrée) et l'Admin peut dépublier (US-033). US-055 reste en P2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-009, US-055</t>
+    <t xml:space="preserve">Autonome au MVP : les partenaires sont onboardés à la main (contrôle à l'entrée) et l'Admin peut dépublier (KAN-59). KAN-28 reste en P2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-26, KAN-28</t>
   </si>
   <si>
     <t xml:space="preserve">Produit</t>
@@ -3217,10 +3217,10 @@
     <t xml:space="preserve">Code • QR • QR + confirmation • code + vérification d'identité</t>
   </si>
   <si>
-    <t xml:space="preserve">QR + saisie de secours, avec confirmation explicite et limitation des tentatives (US-052). La carte est un titre au porteur : le communiquer clairement dans les CGV et sur la page cadeau.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-023, US-026, US-027, US-052</t>
+    <t xml:space="preserve">QR + saisie de secours, avec confirmation explicite et limitation des tentatives (KAN-54). La carte est un titre au porteur : le communiquer clairement dans les CGV et sur la page cadeau.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-45, KAN-49, KAN-50, KAN-54</t>
   </si>
   <si>
     <t xml:space="preserve">Produit / Sécurité</t>
@@ -3238,7 +3238,7 @@
     <t xml:space="preserve">Critères éliminatoires : page hébergée, notification serveur signée, API de consultation de statut, remboursement, environnement de test, délai d'activation. Lancer la consultation dès maintenant (délai d'ouverture du compte marchand).</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018, US-049, US-050</t>
+    <t xml:space="preserve">KAN-38, KAN-42, KAN-43</t>
   </si>
   <si>
     <t xml:space="preserve">Direction / Technique</t>
@@ -3268,7 +3268,7 @@
     <t xml:space="preserve">À trancher contractuellement. Hypothèse du backlog : aucun mouvement à l'expiration, les fonds suivent la règle de reversement (D-11).</t>
   </si>
   <si>
-    <t xml:space="preserve">US-029, US-021, US-030</t>
+    <t xml:space="preserve">KAN-52, KAN-41, KAN-55</t>
   </si>
   <si>
     <t xml:space="preserve">Direction / Juridique</t>
@@ -3283,10 +3283,10 @@
     <t xml:space="preserve">Utilisables • bloquées • remboursées</t>
   </si>
   <si>
-    <t xml:space="preserve">Utilisables par défaut (protection du bénéficiaire) ; l'Admin peut les bloquer au cas par cas (US-051).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-035, US-051</t>
+    <t xml:space="preserve">Utilisables par défaut (protection du bénéficiaire) ; l'Admin peut les bloquer au cas par cas (KAN-53).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-61, KAN-53</t>
   </si>
   <si>
     <t xml:space="preserve">Données personnelles (loi 09-08)</t>
@@ -3301,7 +3301,7 @@
     <t xml:space="preserve">Engager les formalités CNDP avant la mise en production ; documenter l'hébergement (transfert hors Maroc éventuel) ; proposer 24 mois après fin de vie de la carte pour les données personnelles, conservation légale pour les pièces comptables.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-038, US-056, US-057</t>
+    <t xml:space="preserve">KAN-65, KAN-74, KAN-75</t>
   </si>
   <si>
     <t xml:space="preserve">Mise en production</t>
@@ -3322,10 +3322,10 @@
     <t xml:space="preserve">À la vente (net des remboursements) • à l'utilisation</t>
   </si>
   <si>
-    <t xml:space="preserve">Hypothèse du backlog : à la vente, avec déduction des remboursements sur le reversement suivant. « À l'utilisation » protège mieux l'acheteur mais retarde la trésorerie du partenaire et change US-021.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-021, US-031, US-050</t>
+    <t xml:space="preserve">Hypothèse du backlog : à la vente, avec déduction des remboursements sur le reversement suivant. « À l'utilisation » protège mieux l'acheteur mais retarde la trésorerie du partenaire et change KAN-41.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-41, KAN-56, KAN-43</t>
   </si>
   <si>
     <t xml:space="preserve">Direction / Finance</t>
@@ -3340,10 +3340,10 @@
     <t xml:space="preserve">Bornes libres • bornes plateforme</t>
   </si>
   <si>
-    <t xml:space="preserve">50 à 10 000 MAD ; validité 30 à 730 jours, 365 par défaut ; paramétrables plus tard (US-058).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-007, US-058</t>
+    <t xml:space="preserve">50 à 10 000 MAD ; validité 30 à 730 jours, 365 par défaut ; paramétrables plus tard (KAN-62).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-24, KAN-62</t>
   </si>
   <si>
     <t xml:space="preserve">Prévenir l'acheteur de l'utilisation</t>
@@ -3400,7 +3400,7 @@
     <t xml:space="preserve">Lien seulement : limite l'exposition du code (transferts, aperçus) ; le code est sur la page cadeau.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-024, US-023</t>
+    <t xml:space="preserve">KAN-46, KAN-45</t>
   </si>
   <si>
     <t xml:space="preserve">Kadoo | Exigences non fonctionnelles (NFR)</t>
@@ -3520,7 +3520,7 @@
     <t xml:space="preserve">Tests d'intégration sécurité ; revue de configuration.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-001, US-003, US-047</t>
+    <t xml:space="preserve">KAN-17, KAN-19, KAN-20</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-003</t>
@@ -3541,7 +3541,7 @@
     <t xml:space="preserve">Suite « cross-tenant » exécutée à chaque PR : partenaire A tente chaque ressource de B → 404.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-001, US-031, US-054</t>
+    <t xml:space="preserve">KAN-17, KAN-56, KAN-58</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-004</t>
@@ -3562,7 +3562,7 @@
     <t xml:space="preserve">gitleaks en pre-commit et en CI ; revue du schéma.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-004, US-022, US-023, US-047</t>
+    <t xml:space="preserve">KAN-21, KAN-44, KAN-45, KAN-20</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-005</t>
@@ -3583,7 +3583,7 @@
     <t xml:space="preserve">Tests de contrat avec simulateur PSP : signature invalide, rejeu, montant divergent.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018, US-049</t>
+    <t xml:space="preserve">KAN-38, KAN-42</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-006</t>
@@ -3604,7 +3604,7 @@
     <t xml:space="preserve">Tests automatisés dépassant chaque seuil.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-001, US-003, US-052</t>
+    <t xml:space="preserve">KAN-17, KAN-19, KAN-54</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-007</t>
@@ -3643,7 +3643,7 @@
     <t xml:space="preserve">Charges XSS dans les tests E2E ; tests d'upload malveillant.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-016, US-059, US-041</t>
+    <t xml:space="preserve">KAN-35, KAN-29, KAN-68</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-010</t>
@@ -3664,7 +3664,7 @@
     <t xml:space="preserve">Test de concurrence JUnit + Testcontainers PostgreSQL (≥ 50 threads).</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018, US-022, US-036</t>
+    <t xml:space="preserve">KAN-38, KAN-44, KAN-63</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-011</t>
@@ -3700,7 +3700,7 @@
     <t xml:space="preserve">Tests d'intégration avec pannes simulées en cours de transaction.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018, US-020, US-022</t>
+    <t xml:space="preserve">KAN-38, KAN-40, KAN-44</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-013</t>
@@ -3721,7 +3721,7 @@
     <t xml:space="preserve">Injection de pannes avec WireMock (latence, erreurs 5xx).</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018, US-024, US-049</t>
+    <t xml:space="preserve">KAN-38, KAN-46, KAN-42</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-014</t>
@@ -3742,7 +3742,7 @@
     <t xml:space="preserve">Tests unitaires et tests par propriétés (jqwik) sur le calcul de commission.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-019, US-020, US-021</t>
+    <t xml:space="preserve">KAN-39, KAN-40, KAN-41</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-015</t>
@@ -3763,7 +3763,7 @@
     <t xml:space="preserve">Tests autour des dates de changement d'heure et de fin de journée.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-022, US-029, US-030</t>
+    <t xml:space="preserve">KAN-44, KAN-52, KAN-55</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-020</t>
@@ -3787,7 +3787,7 @@
     <t xml:space="preserve">Lighthouse CI en PR avec seuils ; mesure réelle (web-vitals) en production.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-011, US-012, US-023</t>
+    <t xml:space="preserve">KAN-30, KAN-31, KAN-45</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-021</t>
@@ -3823,7 +3823,7 @@
     <t xml:space="preserve">Métrique bout en bout « confirmation → envoi » suivie en recette et en production.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-022, US-024, US-036</t>
+    <t xml:space="preserve">KAN-44, KAN-46, KAN-63</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-023</t>
@@ -3916,7 +3916,7 @@
     <t xml:space="preserve">Tests de panne en préproduction.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018, US-024, US-026</t>
+    <t xml:space="preserve">KAN-38, KAN-46, KAN-49</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-040</t>
@@ -3994,7 +3994,7 @@
     <t xml:space="preserve">Configuration externalisée.</t>
   </si>
   <si>
-    <t xml:space="preserve">Principes 12-factor ; paramètres métier en base (US-058) ; feature flags pour les options en attente de décision (D-04, D-07, D-13).</t>
+    <t xml:space="preserve">Principes 12-factor ; paramètres métier en base (KAN-62) ; feature flags pour les options en attente de décision (D-04, D-07, D-13).</t>
   </si>
   <si>
     <t xml:space="preserve">Variables d'environnement serveur uniquement.</t>
@@ -4006,7 +4006,7 @@
     <t xml:space="preserve">Revue de configuration par environnement.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-055, US-058</t>
+    <t xml:space="preserve">KAN-28, KAN-62</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-045</t>
@@ -4054,7 +4054,7 @@
     <t xml:space="preserve">Revue d'environnement.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-018, US-024</t>
+    <t xml:space="preserve">KAN-38, KAN-46</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-052</t>
@@ -4114,7 +4114,7 @@
     <t xml:space="preserve">Déclenchement simulé de chaque alerte avant go-live.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-024, US-049, US-052</t>
+    <t xml:space="preserve">KAN-46, KAN-42, KAN-54</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-062</t>
@@ -4150,7 +4150,7 @@
     <t xml:space="preserve">Audit automatisé + vérification manuelle sur le parcours nominal.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-011 à US-017, US-023, US-026</t>
+    <t xml:space="preserve">KAN-30, KAN-31, KAN-32, KAN-33, KAN-34, KAN-35, KAN-36, KAN-45, KAN-49</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-071</t>
@@ -4168,7 +4168,7 @@
     <t xml:space="preserve">Recette sur appareils réels Android et iOS.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-011, US-026</t>
+    <t xml:space="preserve">KAN-30, KAN-49</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-072</t>
@@ -4195,7 +4195,7 @@
     <t xml:space="preserve">0 chaîne en dur ; clés manquantes détectées en CI ; URLs localisées /fr, /ar, /en avec hreflang.</t>
   </si>
   <si>
-    <t xml:space="preserve">next-intl (ou équivalent) ; middleware de résolution de langue (US-040).</t>
+    <t xml:space="preserve">next-intl (ou équivalent) ; middleware de résolution de langue (KAN-67).</t>
   </si>
   <si>
     <t xml:space="preserve">MessageSource pour emails et erreurs ; modèles d'email par locale.</t>
@@ -4261,7 +4261,7 @@
     <t xml:space="preserve">Revue juridique avant go-live.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-056, US-057</t>
+    <t xml:space="preserve">KAN-74, KAN-75</t>
   </si>
   <si>
     <t xml:space="preserve">NFR-091</t>
@@ -4291,7 +4291,7 @@
     <t xml:space="preserve">Logs techniques 90 jours ; données personnelles selon D-10 ; audit métier selon obligations comptables.</t>
   </si>
   <si>
-    <t xml:space="preserve">Traitements planifiés de purge et d'anonymisation (US-057).</t>
+    <t xml:space="preserve">Traitements planifiés de purge et d'anonymisation (KAN-75).</t>
   </si>
   <si>
     <t xml:space="preserve">Contrôle trimestriel.</t>
@@ -4399,7 +4399,7 @@
     <t xml:space="preserve">R-02</t>
   </si>
   <si>
-    <t xml:space="preserve">Personas génériques ou erronés : US-004/005 « Admin / Partenaire », US-029 « Partenaire », US-030/031 « Admin / Partenaire », EP12 « Tous / Partenaire / Système ».</t>
+    <t xml:space="preserve">Personas génériques ou erronés : KAN-21/005 « Admin / Partenaire », KAN-52 « Partenaire », KAN-55/031 « Admin / Partenaire », EP12 « Tous / Partenaire / Système ».</t>
   </si>
   <si>
     <t xml:space="preserve">Droits d'accès ambigus pour le développement et la recette.</t>
@@ -4465,7 +4465,7 @@
     <t xml:space="preserve">R-07</t>
   </si>
   <si>
-    <t xml:space="preserve">TransactionCommission (onglet Métier, US-019) et FinancialTransaction (US-020) se recouvrent.</t>
+    <t xml:space="preserve">TransactionCommission (onglet Métier, KAN-39) et FinancialTransaction (KAN-40) se recouvrent.</t>
   </si>
   <si>
     <t xml:space="preserve">Double source de vérité financière.</t>
@@ -4474,7 +4474,7 @@
     <t xml:space="preserve">Fusion dans FinancialTransaction.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-019, US-020</t>
+    <t xml:space="preserve">KAN-39, KAN-40</t>
   </si>
   <si>
     <t xml:space="preserve">R-08</t>
@@ -4510,49 +4510,49 @@
     <t xml:space="preserve">Séquencement</t>
   </si>
   <si>
-    <t xml:space="preserve">US-044 (notifications localisées) en Lot 4 alors que US-002 et US-003 envoient des emails dès le Lot 1.</t>
+    <t xml:space="preserve">KAN-71 (notifications localisées) en Lot 4 alors que KAN-18 et KAN-19 envoient des emails dès le Lot 1.</t>
   </si>
   <si>
     <t xml:space="preserve">Blocage du Lot 1.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-044 déplacée en Lot 1.</t>
+    <t xml:space="preserve">KAN-71 déplacée en Lot 1.</t>
   </si>
   <si>
     <t xml:space="preserve">R-11</t>
   </si>
   <si>
-    <t xml:space="preserve">US-038 (audit) en Lot 5 alors que toutes les US précédentes doivent journaliser.</t>
+    <t xml:space="preserve">KAN-65 (audit) en Lot 5 alors que toutes les US précédentes doivent journaliser.</t>
   </si>
   <si>
     <t xml:space="preserve">Reprise coûteuse en fin de projet.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-038 déplacée en Lot 1.</t>
+    <t xml:space="preserve">KAN-65 déplacée en Lot 1.</t>
   </si>
   <si>
     <t xml:space="preserve">R-12</t>
   </si>
   <si>
-    <t xml:space="preserve">US-036 (confirmation d'achat) en Lot 5 alors qu'elle fait partie du parcours nominal.</t>
+    <t xml:space="preserve">KAN-63 (confirmation d'achat) en Lot 5 alors qu'elle fait partie du parcours nominal.</t>
   </si>
   <si>
     <t xml:space="preserve">Parcours nominal incomplet avant le Lot 5.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-036 déplacée en Lot 4.</t>
+    <t xml:space="preserve">KAN-63 déplacée en Lot 4.</t>
   </si>
   <si>
     <t xml:space="preserve">R-13</t>
   </si>
   <si>
-    <t xml:space="preserve">US-021 (reversements) en P0 Lot 3 alors que le premier reversement n'a lieu qu'à la fin de la première période.</t>
+    <t xml:space="preserve">KAN-41 (reversements) en P0 Lot 3 alors que le premier reversement n'a lieu qu'à la fin de la première période.</t>
   </si>
   <si>
     <t xml:space="preserve">Charge inutile sur le chemin critique.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-021 en P1, Lot 5.</t>
+    <t xml:space="preserve">KAN-41 en P1, Lot 5.</t>
   </si>
   <si>
     <t xml:space="preserve">R-14</t>
@@ -4567,7 +4567,7 @@
     <t xml:space="preserve">HMAC-SHA256 avec clé secrète ; distinction référence publique / code secret.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-022, US-026</t>
+    <t xml:space="preserve">KAN-44, KAN-49</t>
   </si>
   <si>
     <t xml:space="preserve">R-15</t>
@@ -4579,7 +4579,7 @@
     <t xml:space="preserve">Fraude : découverte de cartes valides.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouvelle US-052 (limitation des tentatives).</t>
+    <t xml:space="preserve">Nouvelle KAN-54 (limitation des tentatives).</t>
   </si>
   <si>
     <t xml:space="preserve">R-16</t>
@@ -4591,7 +4591,7 @@
     <t xml:space="preserve">Risque élevé en cas de vol de mot de passe.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouvelle US-047 (MFA Admin).</t>
+    <t xml:space="preserve">Nouvelle KAN-20 (MFA Admin).</t>
   </si>
   <si>
     <t xml:space="preserve">R-17</t>
@@ -4606,7 +4606,7 @@
     <t xml:space="preserve">Commandes PENDING éternelles, KPI faussés.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouvelle US-048.</t>
+    <t xml:space="preserve">Nouvelle KAN-37.</t>
   </si>
   <si>
     <t xml:space="preserve">R-18</t>
@@ -4618,7 +4618,7 @@
     <t xml:space="preserve">Réclamations, perte de confiance.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouvelle US-049 (rapprochement).</t>
+    <t xml:space="preserve">Nouvelle KAN-42 (rapprochement).</t>
   </si>
   <si>
     <t xml:space="preserve">R-19</t>
@@ -4630,10 +4630,10 @@
     <t xml:space="preserve">Pas de réponse aux litiges ; comptes faussés.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouvelles US-050 et US-051 + D-03.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-050, US-051</t>
+    <t xml:space="preserve">Nouvelles KAN-43 et KAN-53 + D-03.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAN-43, KAN-53</t>
   </si>
   <si>
     <t xml:space="preserve">R-20</t>
@@ -4645,7 +4645,7 @@
     <t xml:space="preserve">Cartes payées inutilisables.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouvelle US-053.</t>
+    <t xml:space="preserve">Nouvelle KAN-48.</t>
   </si>
   <si>
     <t xml:space="preserve">R-21</t>
@@ -4657,31 +4657,31 @@
     <t xml:space="preserve">Suivi opérationnel impossible.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouvelle US-054.</t>
+    <t xml:space="preserve">Nouvelle KAN-58.</t>
   </si>
   <si>
     <t xml:space="preserve">R-22</t>
   </si>
   <si>
-    <t xml:space="preserve">US-006 et US-008 supposent des médias « validés » sans US de téléversement.</t>
+    <t xml:space="preserve">KAN-23 et KAN-25 supposent des médias « validés » sans US de téléversement.</t>
   </si>
   <si>
     <t xml:space="preserve">Besoin caché.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouvelle US-059.</t>
+    <t xml:space="preserve">Nouvelle KAN-29.</t>
   </si>
   <si>
     <t xml:space="preserve">R-23</t>
   </si>
   <si>
-    <t xml:space="preserve">US-017 exige un consentement mais aucune US ne gère CGV, mentions légales ni loi 09-08.</t>
+    <t xml:space="preserve">KAN-36 exige un consentement mais aucune US ne gère CGV, mentions légales ni loi 09-08.</t>
   </si>
   <si>
     <t xml:space="preserve">Blocage de la mise en production (PSP, CNDP).</t>
   </si>
   <si>
-    <t xml:space="preserve">Nouvel EP13 : US-056, US-057, US-060 + D-10.</t>
+    <t xml:space="preserve">Nouvel EP13 : KAN-74, KAN-75, KAN-76 + D-10.</t>
   </si>
   <si>
     <t xml:space="preserve">R-24</t>
@@ -4690,7 +4690,7 @@
     <t xml:space="preserve">Règles métier</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuseau et heure d'expiration non définis (US-029).</t>
+    <t xml:space="preserve">Fuseau et heure d'expiration non définis (KAN-52).</t>
   </si>
   <si>
     <t xml:space="preserve">Litiges en caisse le dernier jour.</t>
@@ -4699,7 +4699,7 @@
     <t xml:space="preserve">Expiration à 23:59:59 heure du Maroc.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-022, US-029</t>
+    <t xml:space="preserve">KAN-44, KAN-52</t>
   </si>
   <si>
     <t xml:space="preserve">R-25</t>
@@ -4726,7 +4726,7 @@
     <t xml:space="preserve">Figé à la création de la commande.</t>
   </si>
   <si>
-    <t xml:space="preserve">US-005, US-014, US-019</t>
+    <t xml:space="preserve">KAN-22, KAN-33, KAN-39</t>
   </si>
   <si>
     <t xml:space="preserve">R-27</t>
@@ -4750,13 +4750,13 @@
     <t xml:space="preserve">Client débité sans carte.</t>
   </si>
   <si>
-    <t xml:space="preserve">Accepté, commande PAID (US-048).</t>
+    <t xml:space="preserve">Accepté, commande PAID (KAN-37).</t>
   </si>
   <si>
     <t xml:space="preserve">R-29</t>
   </si>
   <si>
-    <t xml:space="preserve">US-037 : destinataire de la notification d'utilisation non précisé.</t>
+    <t xml:space="preserve">KAN-64 : destinataire de la notification d'utilisation non précisé.</t>
   </si>
   <si>
     <t xml:space="preserve">Choix laissé au développeur.</t>
@@ -5347,7 +5347,7 @@
     <t xml:space="preserve">Pilote</t>
   </si>
   <si>
-    <t xml:space="preserve">2 US du Lot 1 (US-039, US-001) réalisées avec le flux complet, rétrospective, ajustements, puis généralisation.</t>
+    <t xml:space="preserve">2 US du Lot 1 (KAN-66, KAN-17) réalisées avec le flux complet, rétrospective, ajustements, puis généralisation.</t>
   </si>
 </sst>
 </file>

</xml_diff>